<commit_message>
Update member benefits and requirements documents
</commit_message>
<xml_diff>
--- a/需求文档/画原型需求清单.xlsx
+++ b/需求文档/画原型需求清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="11600"/>
+    <workbookView windowWidth="27660" windowHeight="11620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="385">
   <si>
     <t>子系统</t>
   </si>
@@ -80,7 +80,7 @@
     <t>成长值明细</t>
   </si>
   <si>
-    <t>支持会员查询成长值明细，明细需包含成长值获取时间、来源（如消费、签到、评价）、数值</t>
+    <t>支持会员查询成长值明细，明细需包含成长值获取时间、来源（如消费兑成长值、业主身份、居住时长）、数值；每日计算一次，居住时长，为1年时记录一次，为2年时记录一次。不是每天记录一次；有变动才记录，其它类似</t>
   </si>
   <si>
     <t>标签管理</t>
@@ -100,7 +100,7 @@
     <t>详情</t>
   </si>
   <si>
-    <t>会员信息详情查看，展示会员名称、会员ID、手机号、会员等级、会员资产（积分、优惠券、权益）、认证状态、标签等数据</t>
+    <t>会员信息详情查看，展示会员名称、OneID、会员等级、会员资产（积分、优惠券、权益）、认证状态、标签等数据。会员身份信息，支持按来源渠道展示各来源会员ID、所属项目、手机号、证件号；其中手机号、证件号有可能多个</t>
   </si>
   <si>
     <t>导出</t>
@@ -1121,6 +1121,18 @@
   <si>
     <t xml:space="preserve">会员积分中台：积分数据（可用积分、总积分、积分明细）、会员数据（会员等级、成长明细）、获取/消耗积分回传
 </t>
+  </si>
+  <si>
+    <t>会员积分中台，冻解、解冻、黑名单、白名单；帐户的冻解、解冻</t>
+  </si>
+  <si>
+    <t>实时</t>
+  </si>
+  <si>
+    <t>会员注销，用户确认后，无法登陆</t>
+  </si>
+  <si>
+    <t>会员积分中台，预警拦截</t>
   </si>
   <si>
     <t>源：好社区</t>
@@ -1232,7 +1244,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1276,6 +1288,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.75"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -2443,137 +2462,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="57" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="61" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="61" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="62" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="63" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="62" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="64" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="63" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="64" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2886,43 +2905,46 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3461,7 +3483,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H284"/>
+  <dimension ref="A1:H290"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="11" style="1" customWidth="1"/>
@@ -3537,7 +3559,7 @@
       </c>
       <c r="F4" s="51"/>
     </row>
-    <row r="5" s="1" customFormat="1" customHeight="1" spans="1:6">
+    <row r="5" s="1" customFormat="1" ht="40" customHeight="1" spans="1:6">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
       <c r="C5" s="10"/>
@@ -3573,7 +3595,7 @@
       </c>
       <c r="F7" s="51"/>
     </row>
-    <row r="8" s="1" customFormat="1" spans="1:6">
+    <row r="8" s="1" customFormat="1" ht="31" spans="1:6">
       <c r="A8" s="6"/>
       <c r="B8" s="7"/>
       <c r="C8" s="10"/>
@@ -5450,7 +5472,7 @@
       <c r="D158" s="64" t="s">
         <v>311</v>
       </c>
-      <c r="E158" s="108" t="s">
+      <c r="E158" s="106" t="s">
         <v>312</v>
       </c>
       <c r="F158" s="51"/>
@@ -5462,7 +5484,7 @@
       <c r="D159" s="91" t="s">
         <v>313</v>
       </c>
-      <c r="E159" s="109" t="s">
+      <c r="E159" s="107" t="s">
         <v>314</v>
       </c>
       <c r="F159" s="51"/>
@@ -5480,7 +5502,7 @@
       <c r="D160" s="95" t="s">
         <v>317</v>
       </c>
-      <c r="E160" s="110" t="s">
+      <c r="E160" s="108" t="s">
         <v>318</v>
       </c>
       <c r="F160" s="51"/>
@@ -5494,7 +5516,7 @@
       <c r="D161" s="98" t="s">
         <v>320</v>
       </c>
-      <c r="E161" s="110" t="s">
+      <c r="E161" s="108" t="s">
         <v>321</v>
       </c>
       <c r="F161" s="51" t="s">
@@ -5506,7 +5528,7 @@
       <c r="B162" s="93"/>
       <c r="C162" s="99"/>
       <c r="D162" s="100"/>
-      <c r="E162" s="111" t="s">
+      <c r="E162" s="109" t="s">
         <v>323</v>
       </c>
       <c r="F162" s="51" t="s">
@@ -5518,7 +5540,7 @@
       <c r="B163" s="93"/>
       <c r="C163" s="99"/>
       <c r="D163" s="100"/>
-      <c r="E163" s="111" t="s">
+      <c r="E163" s="109" t="s">
         <v>325</v>
       </c>
       <c r="F163" s="51" t="s">
@@ -5530,7 +5552,7 @@
       <c r="B164" s="93"/>
       <c r="C164" s="101"/>
       <c r="D164" s="102"/>
-      <c r="E164" s="110" t="s">
+      <c r="E164" s="108" t="s">
         <v>326</v>
       </c>
       <c r="F164" s="51"/>
@@ -5544,7 +5566,7 @@
       <c r="D165" s="104" t="s">
         <v>328</v>
       </c>
-      <c r="E165" s="112" t="s">
+      <c r="E165" s="110" t="s">
         <v>329</v>
       </c>
       <c r="F165" s="51"/>
@@ -5556,7 +5578,7 @@
       <c r="D166" s="104" t="s">
         <v>328</v>
       </c>
-      <c r="E166" s="112" t="s">
+      <c r="E166" s="110" t="s">
         <v>330</v>
       </c>
       <c r="F166" s="51" t="s">
@@ -5570,7 +5592,7 @@
       <c r="D167" s="104" t="s">
         <v>320</v>
       </c>
-      <c r="E167" s="112" t="s">
+      <c r="E167" s="110" t="s">
         <v>331</v>
       </c>
       <c r="F167" s="51"/>
@@ -5584,7 +5606,7 @@
       <c r="D168" s="104" t="s">
         <v>328</v>
       </c>
-      <c r="E168" s="112" t="s">
+      <c r="E168" s="110" t="s">
         <v>333</v>
       </c>
       <c r="F168" s="51"/>
@@ -5596,7 +5618,7 @@
       <c r="D169" s="104" t="s">
         <v>328</v>
       </c>
-      <c r="E169" s="112" t="s">
+      <c r="E169" s="110" t="s">
         <v>334</v>
       </c>
       <c r="F169" s="51" t="s">
@@ -5610,7 +5632,7 @@
       <c r="D170" s="104" t="s">
         <v>320</v>
       </c>
-      <c r="E170" s="112" t="s">
+      <c r="E170" s="110" t="s">
         <v>335</v>
       </c>
       <c r="F170" s="51"/>
@@ -5624,7 +5646,7 @@
       <c r="D171" s="105" t="s">
         <v>320</v>
       </c>
-      <c r="E171" s="112" t="s">
+      <c r="E171" s="110" t="s">
         <v>337</v>
       </c>
       <c r="F171" s="51" t="s">
@@ -5638,7 +5660,7 @@
       <c r="D172" s="105" t="s">
         <v>320</v>
       </c>
-      <c r="E172" s="112" t="s">
+      <c r="E172" s="110" t="s">
         <v>338</v>
       </c>
       <c r="F172" s="51" t="s">
@@ -5652,7 +5674,7 @@
       <c r="D173" s="105" t="s">
         <v>320</v>
       </c>
-      <c r="E173" s="112" t="s">
+      <c r="E173" s="110" t="s">
         <v>340</v>
       </c>
       <c r="F173" s="51"/>
@@ -5664,7 +5686,7 @@
       <c r="D174" s="105" t="s">
         <v>328</v>
       </c>
-      <c r="E174" s="112" t="s">
+      <c r="E174" s="110" t="s">
         <v>341</v>
       </c>
       <c r="F174" s="51" t="s">
@@ -5678,7 +5700,7 @@
       <c r="D175" s="105" t="s">
         <v>343</v>
       </c>
-      <c r="E175" s="112" t="s">
+      <c r="E175" s="110" t="s">
         <v>344</v>
       </c>
       <c r="F175" s="51" t="s">
@@ -5692,7 +5714,7 @@
       <c r="D176" s="105" t="s">
         <v>320</v>
       </c>
-      <c r="E176" s="112" t="s">
+      <c r="E176" s="110" t="s">
         <v>345</v>
       </c>
       <c r="F176" s="51"/>
@@ -5706,7 +5728,7 @@
       <c r="D177" s="105" t="s">
         <v>346</v>
       </c>
-      <c r="E177" s="113" t="s">
+      <c r="E177" s="111" t="s">
         <v>347</v>
       </c>
       <c r="F177" s="51" t="s">
@@ -5718,226 +5740,216 @@
       <c r="B178" s="93"/>
       <c r="C178" s="103"/>
       <c r="D178" s="105"/>
-      <c r="E178" s="112" t="s">
-        <v>318</v>
-      </c>
-      <c r="F178" s="51"/>
+      <c r="E178" s="111" t="s">
+        <v>348</v>
+      </c>
+      <c r="F178" s="112" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="179" s="1" customFormat="1" spans="1:6">
       <c r="A179" s="96"/>
       <c r="B179" s="93"/>
-      <c r="C179" s="103" t="s">
-        <v>348</v>
-      </c>
-      <c r="D179" s="105" t="s">
-        <v>320</v>
-      </c>
-      <c r="E179" s="112" t="s">
-        <v>349</v>
-      </c>
-      <c r="F179" s="51" t="s">
-        <v>322</v>
-      </c>
+      <c r="C179" s="103"/>
+      <c r="D179" s="105"/>
+      <c r="E179" s="111" t="s">
+        <v>350</v>
+      </c>
+      <c r="F179" s="112"/>
     </row>
     <row r="180" s="1" customFormat="1" spans="1:6">
       <c r="A180" s="96"/>
       <c r="B180" s="93"/>
       <c r="C180" s="103"/>
       <c r="D180" s="105"/>
-      <c r="E180" s="112" t="s">
-        <v>340</v>
-      </c>
-      <c r="F180" s="51"/>
+      <c r="E180" s="111" t="s">
+        <v>351</v>
+      </c>
+      <c r="F180" s="51" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="181" s="1" customFormat="1" spans="1:6">
       <c r="A181" s="96"/>
       <c r="B181" s="93"/>
       <c r="C181" s="103"/>
       <c r="D181" s="105"/>
-      <c r="E181" s="112" t="s">
-        <v>350</v>
-      </c>
-      <c r="F181" s="51" t="s">
-        <v>322</v>
-      </c>
+      <c r="E181" s="110" t="s">
+        <v>318</v>
+      </c>
+      <c r="F181" s="51"/>
     </row>
     <row r="182" s="1" customFormat="1" spans="1:6">
       <c r="A182" s="96"/>
       <c r="B182" s="93"/>
-      <c r="C182" s="103"/>
-      <c r="D182" s="105"/>
-      <c r="E182" s="112" t="s">
-        <v>351</v>
-      </c>
-      <c r="F182" s="51"/>
+      <c r="C182" s="103" t="s">
+        <v>352</v>
+      </c>
+      <c r="D182" s="105" t="s">
+        <v>320</v>
+      </c>
+      <c r="E182" s="110" t="s">
+        <v>353</v>
+      </c>
+      <c r="F182" s="51" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="183" s="1" customFormat="1" spans="1:6">
       <c r="A183" s="96"/>
       <c r="B183" s="93"/>
       <c r="C183" s="103"/>
       <c r="D183" s="105"/>
-      <c r="E183" s="112" t="s">
-        <v>345</v>
+      <c r="E183" s="110" t="s">
+        <v>340</v>
       </c>
       <c r="F183" s="51"/>
     </row>
-    <row r="184" s="1" customFormat="1" ht="34" spans="1:8">
+    <row r="184" s="1" customFormat="1" spans="1:6">
       <c r="A184" s="96"/>
       <c r="B184" s="93"/>
-      <c r="C184" s="103" t="s">
-        <v>316</v>
-      </c>
-      <c r="D184" s="105" t="s">
-        <v>352</v>
-      </c>
-      <c r="E184" s="112" t="s">
-        <v>353</v>
+      <c r="C184" s="103"/>
+      <c r="D184" s="105"/>
+      <c r="E184" s="110" t="s">
+        <v>354</v>
       </c>
       <c r="F184" s="51" t="s">
         <v>322</v>
       </c>
-      <c r="G184" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="H184" s="114" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="185" s="1" customFormat="1" spans="1:8">
+    </row>
+    <row r="185" s="1" customFormat="1" spans="1:6">
       <c r="A185" s="96"/>
       <c r="B185" s="93"/>
       <c r="C185" s="103"/>
       <c r="D185" s="105"/>
-      <c r="E185" s="112" t="s">
-        <v>318</v>
+      <c r="E185" s="110" t="s">
+        <v>355</v>
       </c>
       <c r="F185" s="51"/>
-      <c r="G185" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="H185" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="186" s="1" customFormat="1" spans="1:8">
+    </row>
+    <row r="186" s="1" customFormat="1" spans="1:6">
       <c r="A186" s="96"/>
       <c r="B186" s="93"/>
-      <c r="C186" s="103" t="s">
-        <v>358</v>
-      </c>
-      <c r="D186" s="105" t="s">
-        <v>320</v>
-      </c>
-      <c r="E186" s="112" t="s">
-        <v>359</v>
+      <c r="C186" s="103"/>
+      <c r="D186" s="105"/>
+      <c r="E186" s="110" t="s">
+        <v>345</v>
       </c>
       <c r="F186" s="51"/>
-      <c r="H186" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="187" s="1" customFormat="1" spans="1:8">
+    </row>
+    <row r="187" s="1" customFormat="1" ht="34" spans="1:8">
       <c r="A187" s="96"/>
       <c r="B187" s="93"/>
-      <c r="C187" s="106" t="s">
-        <v>361</v>
+      <c r="C187" s="103" t="s">
+        <v>316</v>
       </c>
       <c r="D187" s="105" t="s">
-        <v>320</v>
-      </c>
-      <c r="E187" s="112" t="s">
-        <v>362</v>
-      </c>
-      <c r="F187" s="51"/>
-      <c r="H187" s="1" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="188" s="1" customFormat="1" spans="1:6">
+        <v>356</v>
+      </c>
+      <c r="E187" s="110" t="s">
+        <v>357</v>
+      </c>
+      <c r="F187" s="51" t="s">
+        <v>322</v>
+      </c>
+      <c r="G187" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="H187" s="113" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="188" s="1" customFormat="1" spans="1:8">
       <c r="A188" s="96"/>
       <c r="B188" s="93"/>
-      <c r="C188" s="107"/>
-      <c r="D188" s="105" t="s">
-        <v>320</v>
-      </c>
-      <c r="E188" s="112" t="s">
-        <v>364</v>
+      <c r="C188" s="103"/>
+      <c r="D188" s="105"/>
+      <c r="E188" s="111" t="s">
+        <v>348</v>
       </c>
       <c r="F188" s="51"/>
-    </row>
-    <row r="189" s="1" customFormat="1" spans="1:6">
+      <c r="H188" s="113"/>
+    </row>
+    <row r="189" s="1" customFormat="1" spans="1:8">
       <c r="A189" s="96"/>
       <c r="B189" s="93"/>
-      <c r="C189" s="103" t="s">
-        <v>316</v>
-      </c>
-      <c r="D189" s="105" t="s">
-        <v>365</v>
-      </c>
-      <c r="E189" s="112" t="s">
-        <v>353</v>
+      <c r="C189" s="103"/>
+      <c r="D189" s="105"/>
+      <c r="E189" s="111" t="s">
+        <v>351</v>
       </c>
       <c r="F189" s="51"/>
+      <c r="H189" s="113"/>
     </row>
     <row r="190" s="1" customFormat="1" spans="1:6">
       <c r="A190" s="96"/>
       <c r="B190" s="93"/>
       <c r="C190" s="103"/>
       <c r="D190" s="105"/>
-      <c r="E190" s="112" t="s">
-        <v>340</v>
+      <c r="E190" s="110" t="s">
+        <v>350</v>
       </c>
       <c r="F190" s="51"/>
     </row>
-    <row r="191" s="1" customFormat="1" spans="1:6">
+    <row r="191" s="1" customFormat="1" spans="1:8">
       <c r="A191" s="96"/>
       <c r="B191" s="93"/>
       <c r="C191" s="103"/>
       <c r="D191" s="105"/>
-      <c r="E191" s="112" t="s">
+      <c r="E191" s="110" t="s">
         <v>318</v>
       </c>
       <c r="F191" s="51"/>
-    </row>
-    <row r="192" s="1" customFormat="1" spans="1:6">
+      <c r="G191" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="H191" s="1" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="192" s="1" customFormat="1" spans="1:8">
       <c r="A192" s="96"/>
       <c r="B192" s="93"/>
       <c r="C192" s="103" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="D192" s="105" t="s">
-        <v>367</v>
-      </c>
-      <c r="E192" s="112" t="s">
-        <v>368</v>
+        <v>320</v>
+      </c>
+      <c r="E192" s="110" t="s">
+        <v>363</v>
       </c>
       <c r="F192" s="51"/>
-    </row>
-    <row r="193" s="1" customFormat="1" spans="1:6">
+      <c r="H192" s="1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="193" s="1" customFormat="1" spans="1:8">
       <c r="A193" s="96"/>
       <c r="B193" s="93"/>
-      <c r="C193" s="103" t="s">
-        <v>316</v>
+      <c r="C193" s="114" t="s">
+        <v>365</v>
       </c>
       <c r="D193" s="105" t="s">
-        <v>369</v>
-      </c>
-      <c r="E193" s="112" t="s">
-        <v>370</v>
+        <v>320</v>
+      </c>
+      <c r="E193" s="110" t="s">
+        <v>366</v>
       </c>
       <c r="F193" s="51"/>
+      <c r="H193" s="1" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="194" s="1" customFormat="1" spans="1:6">
       <c r="A194" s="96"/>
       <c r="B194" s="93"/>
-      <c r="C194" s="115" t="s">
-        <v>371</v>
-      </c>
+      <c r="C194" s="115"/>
       <c r="D194" s="105" t="s">
-        <v>372</v>
-      </c>
-      <c r="E194" s="112" t="s">
-        <v>351</v>
+        <v>320</v>
+      </c>
+      <c r="E194" s="110" t="s">
+        <v>368</v>
       </c>
       <c r="F194" s="51"/>
     </row>
@@ -5948,86 +5960,144 @@
         <v>316</v>
       </c>
       <c r="D195" s="105" t="s">
+        <v>369</v>
+      </c>
+      <c r="E195" s="110" t="s">
+        <v>357</v>
+      </c>
+      <c r="F195" s="51"/>
+    </row>
+    <row r="196" s="1" customFormat="1" spans="1:6">
+      <c r="A196" s="96"/>
+      <c r="B196" s="93"/>
+      <c r="C196" s="103"/>
+      <c r="D196" s="105"/>
+      <c r="E196" s="110" t="s">
+        <v>340</v>
+      </c>
+      <c r="F196" s="51"/>
+    </row>
+    <row r="197" s="1" customFormat="1" spans="1:6">
+      <c r="A197" s="96"/>
+      <c r="B197" s="93"/>
+      <c r="C197" s="103"/>
+      <c r="D197" s="105"/>
+      <c r="E197" s="110" t="s">
+        <v>318</v>
+      </c>
+      <c r="F197" s="51"/>
+    </row>
+    <row r="198" s="1" customFormat="1" spans="1:6">
+      <c r="A198" s="96"/>
+      <c r="B198" s="93"/>
+      <c r="C198" s="103" t="s">
+        <v>370</v>
+      </c>
+      <c r="D198" s="105" t="s">
+        <v>371</v>
+      </c>
+      <c r="E198" s="110" t="s">
+        <v>372</v>
+      </c>
+      <c r="F198" s="51"/>
+    </row>
+    <row r="199" s="1" customFormat="1" spans="1:6">
+      <c r="A199" s="96"/>
+      <c r="B199" s="93"/>
+      <c r="C199" s="103" t="s">
+        <v>316</v>
+      </c>
+      <c r="D199" s="105" t="s">
         <v>373</v>
       </c>
-      <c r="E195" s="112" t="s">
+      <c r="E199" s="110" t="s">
         <v>374</v>
       </c>
-      <c r="F195" s="51"/>
-    </row>
-    <row r="196" s="1" customFormat="1" spans="1:6">
-      <c r="A196" s="116"/>
-      <c r="B196" s="93"/>
-      <c r="C196" s="117" t="s">
+      <c r="F199" s="51"/>
+    </row>
+    <row r="200" s="1" customFormat="1" spans="1:6">
+      <c r="A200" s="96"/>
+      <c r="B200" s="93"/>
+      <c r="C200" s="116" t="s">
         <v>375</v>
       </c>
-      <c r="D196" s="118" t="s">
-        <v>375</v>
-      </c>
-      <c r="E196" s="120" t="s">
+      <c r="D200" s="105" t="s">
         <v>376</v>
       </c>
-      <c r="F196" s="51"/>
-    </row>
-    <row r="197" s="1" customFormat="1" spans="1:6">
-      <c r="A197" s="51" t="s">
+      <c r="E200" s="110" t="s">
+        <v>355</v>
+      </c>
+      <c r="F200" s="51"/>
+    </row>
+    <row r="201" s="1" customFormat="1" spans="1:6">
+      <c r="A201" s="96"/>
+      <c r="B201" s="93"/>
+      <c r="C201" s="103" t="s">
+        <v>316</v>
+      </c>
+      <c r="D201" s="105" t="s">
         <v>377</v>
       </c>
-      <c r="B197" s="51" t="s">
-        <v>377</v>
-      </c>
-      <c r="C197" s="119" t="s">
+      <c r="E201" s="110" t="s">
         <v>378</v>
       </c>
-      <c r="D197" s="51" t="s">
+      <c r="F201" s="51"/>
+    </row>
+    <row r="202" s="1" customFormat="1" spans="1:6">
+      <c r="A202" s="117"/>
+      <c r="B202" s="93"/>
+      <c r="C202" s="118" t="s">
         <v>379</v>
       </c>
-      <c r="E197" s="51"/>
-      <c r="F197" s="51"/>
-    </row>
-    <row r="198" s="1" customFormat="1" spans="1:6">
-      <c r="A198" s="51"/>
-      <c r="B198" s="51"/>
-      <c r="C198" s="119"/>
-      <c r="D198" s="51" t="s">
+      <c r="D202" s="119" t="s">
+        <v>379</v>
+      </c>
+      <c r="E202" s="121" t="s">
         <v>380</v>
       </c>
-      <c r="E198" s="51"/>
-      <c r="F198" s="51"/>
-    </row>
-    <row r="199" s="1" customFormat="1" spans="1:6">
-      <c r="A199" s="51"/>
-      <c r="B199" s="51"/>
-      <c r="C199" s="119"/>
-      <c r="D199" s="51"/>
-      <c r="E199" s="51"/>
-      <c r="F199" s="51"/>
-    </row>
-    <row r="200" s="1" customFormat="1" spans="1:6">
-      <c r="A200" s="51"/>
-      <c r="B200" s="51"/>
-      <c r="C200" s="119"/>
-      <c r="D200" s="51"/>
-      <c r="E200" s="51"/>
-      <c r="F200" s="51"/>
-    </row>
-    <row r="201" s="1" customFormat="1" spans="3:3">
-      <c r="C201" s="3"/>
-    </row>
-    <row r="202" s="1" customFormat="1" spans="3:3">
-      <c r="C202" s="3"/>
-    </row>
-    <row r="203" s="1" customFormat="1" spans="3:3">
-      <c r="C203" s="3"/>
-    </row>
-    <row r="204" s="1" customFormat="1" spans="3:3">
-      <c r="C204" s="3"/>
-    </row>
-    <row r="205" s="1" customFormat="1" spans="3:3">
-      <c r="C205" s="3"/>
-    </row>
-    <row r="206" s="1" customFormat="1" spans="3:3">
-      <c r="C206" s="3"/>
+      <c r="F202" s="51"/>
+    </row>
+    <row r="203" s="1" customFormat="1" spans="1:6">
+      <c r="A203" s="51" t="s">
+        <v>381</v>
+      </c>
+      <c r="B203" s="51" t="s">
+        <v>381</v>
+      </c>
+      <c r="C203" s="120" t="s">
+        <v>382</v>
+      </c>
+      <c r="D203" s="51" t="s">
+        <v>383</v>
+      </c>
+      <c r="E203" s="51"/>
+      <c r="F203" s="51"/>
+    </row>
+    <row r="204" s="1" customFormat="1" spans="1:6">
+      <c r="A204" s="51"/>
+      <c r="B204" s="51"/>
+      <c r="C204" s="120"/>
+      <c r="D204" s="51" t="s">
+        <v>384</v>
+      </c>
+      <c r="E204" s="51"/>
+      <c r="F204" s="51"/>
+    </row>
+    <row r="205" s="1" customFormat="1" spans="1:6">
+      <c r="A205" s="51"/>
+      <c r="B205" s="51"/>
+      <c r="C205" s="120"/>
+      <c r="D205" s="51"/>
+      <c r="E205" s="51"/>
+      <c r="F205" s="51"/>
+    </row>
+    <row r="206" s="1" customFormat="1" spans="1:6">
+      <c r="A206" s="51"/>
+      <c r="B206" s="51"/>
+      <c r="C206" s="120"/>
+      <c r="D206" s="51"/>
+      <c r="E206" s="51"/>
+      <c r="F206" s="51"/>
     </row>
     <row r="207" s="1" customFormat="1" spans="3:3">
       <c r="C207" s="3"/>
@@ -6262,13 +6332,31 @@
     </row>
     <row r="284" s="1" customFormat="1" spans="3:3">
       <c r="C284" s="3"/>
+    </row>
+    <row r="285" s="1" customFormat="1" spans="3:3">
+      <c r="C285" s="3"/>
+    </row>
+    <row r="286" s="1" customFormat="1" spans="3:3">
+      <c r="C286" s="3"/>
+    </row>
+    <row r="287" s="1" customFormat="1" spans="3:3">
+      <c r="C287" s="3"/>
+    </row>
+    <row r="288" s="1" customFormat="1" spans="3:3">
+      <c r="C288" s="3"/>
+    </row>
+    <row r="289" s="1" customFormat="1" spans="3:3">
+      <c r="C289" s="3"/>
+    </row>
+    <row r="290" s="1" customFormat="1" spans="3:3">
+      <c r="C290" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="95">
     <mergeCell ref="A2:A89"/>
     <mergeCell ref="A90:A135"/>
     <mergeCell ref="A136:A159"/>
-    <mergeCell ref="A160:A196"/>
+    <mergeCell ref="A160:A202"/>
     <mergeCell ref="B2:B20"/>
     <mergeCell ref="B21:B38"/>
     <mergeCell ref="B39:B54"/>
@@ -6288,7 +6376,7 @@
     <mergeCell ref="B144:B148"/>
     <mergeCell ref="B149:B153"/>
     <mergeCell ref="B154:B159"/>
-    <mergeCell ref="B160:B196"/>
+    <mergeCell ref="B160:B202"/>
     <mergeCell ref="C2:C9"/>
     <mergeCell ref="C10:C14"/>
     <mergeCell ref="C15:C18"/>
@@ -6330,11 +6418,11 @@
     <mergeCell ref="C165:C167"/>
     <mergeCell ref="C168:C170"/>
     <mergeCell ref="C171:C176"/>
-    <mergeCell ref="C177:C178"/>
-    <mergeCell ref="C179:C183"/>
-    <mergeCell ref="C184:C185"/>
-    <mergeCell ref="C187:C188"/>
-    <mergeCell ref="C189:C191"/>
+    <mergeCell ref="C177:C181"/>
+    <mergeCell ref="C182:C186"/>
+    <mergeCell ref="C187:C191"/>
+    <mergeCell ref="C193:C194"/>
+    <mergeCell ref="C195:C197"/>
     <mergeCell ref="D16:D18"/>
     <mergeCell ref="D30:D31"/>
     <mergeCell ref="D34:D36"/>
@@ -6356,10 +6444,10 @@
     <mergeCell ref="D150:D152"/>
     <mergeCell ref="D154:D155"/>
     <mergeCell ref="D161:D164"/>
-    <mergeCell ref="D177:D178"/>
-    <mergeCell ref="D179:D183"/>
-    <mergeCell ref="D184:D185"/>
-    <mergeCell ref="D189:D191"/>
+    <mergeCell ref="D177:D181"/>
+    <mergeCell ref="D182:D186"/>
+    <mergeCell ref="D187:D191"/>
+    <mergeCell ref="D195:D197"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>